<commit_message>
Add capillary pressure import from SCAL (Leverett J)
- read Pc tables (Sw or mercury saturation + Pc) from the same reports:
  units from the header (psi, kPa, MPa, bar, atm, kgf/cm2), lab system from a
  column, sheet or file name (mercury-air, air-brine, oil-brine)
- convert lab Pc to reservoir oil-water Pc with sigma*cos(theta) ratios,
  compute Leverett J per point with sample k and porosity
- fit J = a*Sn^-b to pooled normalized points per rock type -> LeverettJ in the
  rock type (Brooks-Corey fallback without k/phi), Pcmax from the data
- QC plot (lab Pc, J fit, reservoir Pcow with height above FWL), lab Pc overlay
  for the editor (--lab-pc), summary with entry height above FWL
- CLI flags --pc-lab-units, --pc-system, --ift-res, --theta-res, --pc-units, --drho
- MPa accepted as Pc units; example report gains MICP, centrifuge and porous plate data

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TeuneQWQ2dg2q4itUSZbGc
</commit_message>
<xml_diff>
--- a/examples/scal_lab_report.xlsx
+++ b/examples/scal_lab_report.xlsx
@@ -16,14 +16,19 @@
     <sheet name="202" sheetId="7" r:id="rId7"/>
     <sheet name="203" sheetId="8" r:id="rId8"/>
     <sheet name="204" sheetId="9" r:id="rId9"/>
-    <sheet name="Газ-нефть" sheetId="10" r:id="rId10"/>
+    <sheet name="101 MICP" sheetId="10" r:id="rId10"/>
+    <sheet name="102 MICP" sheetId="11" r:id="rId11"/>
+    <sheet name="Рк 202 центрифуга" sheetId="12" r:id="rId12"/>
+    <sheet name="Рк 203 центрифуга" sheetId="13" r:id="rId13"/>
+    <sheet name="Капилляриметрия" sheetId="14" r:id="rId14"/>
+    <sheet name="Газ-нефть" sheetId="15" r:id="rId15"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="33">
   <si>
     <t>Отчёт: специальные исследования керна (ОФП), синтетический пример</t>
   </si>
@@ -80,6 +85,39 @@
   </si>
   <si>
     <t>Образец 204: вытеснение нефти водой (USS)</t>
+  </si>
+  <si>
+    <t>101 MICP: капиллярное давление</t>
+  </si>
+  <si>
+    <t>SHg, %</t>
+  </si>
+  <si>
+    <t>Pc, psi</t>
+  </si>
+  <si>
+    <t>102 MICP: капиллярное давление</t>
+  </si>
+  <si>
+    <t>Рк 202 центрифуга: капиллярное давление</t>
+  </si>
+  <si>
+    <t>Кв, д.ед.</t>
+  </si>
+  <si>
+    <t>Рк, МПа</t>
+  </si>
+  <si>
+    <t>Рк 203 центрифуга: капиллярное давление</t>
+  </si>
+  <si>
+    <t>Система</t>
+  </si>
+  <si>
+    <t>Рк, атм</t>
+  </si>
+  <si>
+    <t>газ-вода</t>
   </si>
   <si>
     <t>Sg, д.ед.</t>
@@ -588,6 +626,464 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="B4">
+        <v>1291.483</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="B5">
+        <v>1359.867</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6">
+        <v>72.59999999999999</v>
+      </c>
+      <c r="B6">
+        <v>375.928</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7">
+        <v>66.22</v>
+      </c>
+      <c r="B7">
+        <v>79.797</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8">
+        <v>59.85</v>
+      </c>
+      <c r="B8">
+        <v>41.003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9">
+        <v>53.47</v>
+      </c>
+      <c r="B9">
+        <v>26.114</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10">
+        <v>47.09</v>
+      </c>
+      <c r="B10">
+        <v>19.632</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11">
+        <v>40.72</v>
+      </c>
+      <c r="B11">
+        <v>14.731</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12">
+        <v>34.34</v>
+      </c>
+      <c r="B12">
+        <v>12.224</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13">
+        <v>27.97</v>
+      </c>
+      <c r="B13">
+        <v>9.119</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14">
+        <v>21.59</v>
+      </c>
+      <c r="B14">
+        <v>8.887</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4">
+        <v>85.3</v>
+      </c>
+      <c r="B4">
+        <v>925.667</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5">
+        <v>80.3</v>
+      </c>
+      <c r="B5">
+        <v>954.5410000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6">
+        <v>74.3</v>
+      </c>
+      <c r="B6">
+        <v>270.605</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7">
+        <v>67.64</v>
+      </c>
+      <c r="B7">
+        <v>58.563</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8">
+        <v>60.97</v>
+      </c>
+      <c r="B8">
+        <v>30.628</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9">
+        <v>54.31</v>
+      </c>
+      <c r="B9">
+        <v>19.907</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10">
+        <v>47.64</v>
+      </c>
+      <c r="B10">
+        <v>13.73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11">
+        <v>40.98</v>
+      </c>
+      <c r="B11">
+        <v>10.571</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12">
+        <v>34.31</v>
+      </c>
+      <c r="B12">
+        <v>8.778</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13">
+        <v>27.65</v>
+      </c>
+      <c r="B13">
+        <v>6.837</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14">
+        <v>20.99</v>
+      </c>
+      <c r="B14">
+        <v>5.65</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4">
+        <v>0.389</v>
+      </c>
+      <c r="B4">
+        <v>0.6221100000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5">
+        <v>0.4403</v>
+      </c>
+      <c r="B5">
+        <v>0.24049</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6">
+        <v>0.4916</v>
+      </c>
+      <c r="B6">
+        <v>0.13971</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7">
+        <v>0.5427999999999999</v>
+      </c>
+      <c r="B7">
+        <v>0.10441</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8">
+        <v>0.5941</v>
+      </c>
+      <c r="B8">
+        <v>0.08180999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9">
+        <v>0.6454</v>
+      </c>
+      <c r="B9">
+        <v>0.06442000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10">
+        <v>0.6967</v>
+      </c>
+      <c r="B10">
+        <v>0.05337</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4">
+        <v>0.339</v>
+      </c>
+      <c r="B4">
+        <v>0.57729</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5">
+        <v>0.404</v>
+      </c>
+      <c r="B5">
+        <v>0.20653</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6">
+        <v>0.469</v>
+      </c>
+      <c r="B6">
+        <v>0.11625</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7">
+        <v>0.534</v>
+      </c>
+      <c r="B7">
+        <v>0.07974000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8">
+        <v>0.599</v>
+      </c>
+      <c r="B8">
+        <v>0.06379</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9">
+        <v>0.6641</v>
+      </c>
+      <c r="B9">
+        <v>0.05209</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10">
+        <v>0.7291</v>
+      </c>
+      <c r="B10">
+        <v>0.04177</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2">
+        <v>104</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2">
+        <v>22.1</v>
+      </c>
+      <c r="D2">
+        <v>2.0468</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="C3">
+        <v>32.8</v>
+      </c>
+      <c r="D3">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="C4">
+        <v>43.5</v>
+      </c>
+      <c r="D4">
+        <v>0.1304</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="C5">
+        <v>54.2</v>
+      </c>
+      <c r="D5">
+        <v>0.0793</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="C6">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="D6">
+        <v>0.0588</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="C7">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="D7">
+        <v>0.0446</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -596,13 +1092,13 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="C1" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:4">

</xml_diff>